<commit_message>
Added Baseline folder, Updated RAD test cases for Motor Fuel Floor Tax
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/UM-Data-Prod.xlsx
+++ b/KatalonData/Bootstrap/UM-Data-Prod.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="170">
   <si>
     <t>Notes</t>
   </si>
@@ -527,6 +527,30 @@
   </si>
   <si>
     <t>Tue Jun 16 23:43:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 19:53:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 15:58:52 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:02:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:03:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:03:21 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:03:42 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:04:05 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:04:33 EDT 2026</t>
   </si>
 </sst>
 </file>
@@ -899,7 +923,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E041308-6561-4EE5-9DD4-5DDA2695E487}">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.5546875" collapsed="true"/>
@@ -963,16 +987,16 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="1">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="1">
+        <v>166</v>
+      </c>
+      <c r="C2" t="s" s="1">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="1">
         <v>157</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -987,10 +1011,10 @@
       <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="1">
         <v>15</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="1">
         <v>15</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -998,13 +1022,13 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
       <c r="K4" s="2"/>
-      <c r="L4"/>
-      <c r="M4"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -1017,7 +1041,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D7D96D8-F32A-42CB-8719-B4A22D28EC0D}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultColWidth="19.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.5546875" collapsed="true"/>
@@ -1069,16 +1093,16 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="1">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="1">
+        <v>167</v>
+      </c>
+      <c r="C2" t="s" s="1">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="1">
         <v>158</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -1095,64 +1119,64 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3"/>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5"/>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7"/>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8"/>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9"/>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10"/>
-      <c r="B10"/>
-      <c r="C10"/>
-      <c r="D10"/>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11"/>
-      <c r="B11"/>
-      <c r="C11"/>
-      <c r="D11"/>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12"/>
-      <c r="B12"/>
-      <c r="C12"/>
-      <c r="D12"/>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13"/>
-      <c r="B13"/>
-      <c r="C13"/>
-      <c r="D13"/>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -1165,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28ECF6F8-94D7-41D5-B6FF-650248E68667}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="8" customWidth="true" width="30.109375" collapsed="true"/>
@@ -1216,16 +1240,16 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="C2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>159</v>
       </c>
       <c r="E2" s="1"/>
@@ -1243,10 +1267,10 @@
       <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>15</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -1260,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5380E685-D2A4-4DCA-A76F-EFBA3980BCE7}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" customWidth="true" width="22.33203125" collapsed="true"/>
@@ -1271,81 +1295,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" t="s" s="0">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="C2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>160</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="0">
         <v>13</v>
       </c>
     </row>
@@ -1356,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ECF5EAC-3F98-4000-BEA2-335F903FE34F}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="9" customWidth="true" width="22.0" collapsed="true"/>
@@ -1401,16 +1425,16 @@
       </c>
     </row>
     <row ht="28.8" r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="0">
+        <v>163</v>
+      </c>
+      <c r="C2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>161</v>
       </c>
       <c r="E2" s="1"/>
@@ -1439,7 +1463,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A53983D-C89C-4548-8A02-C36CB8EC5C28}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="3" width="6.5546875" collapsed="true"/>
@@ -1480,16 +1504,16 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="3">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s" s="3">
+        <v>164</v>
+      </c>
+      <c r="C2" t="s" s="3">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="3">
         <v>155</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -1506,22 +1530,22 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3"/>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5"/>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -1530,7 +1554,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCABF931-E9E5-40BE-B844-C9FC3C47A38B}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" style="3" width="9.109375" collapsed="true"/>
@@ -1571,16 +1595,16 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="3">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="3">
+        <v>165</v>
+      </c>
+      <c r="C2" t="s" s="3">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="3">
         <v>156</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -1597,22 +1621,22 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3"/>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5"/>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Online Reporting TestCases Done
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/UM-Data-Prod.xlsx
+++ b/KatalonData/Bootstrap/UM-Data-Prod.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t476046\Documents\VPS-Katalon-feature-VRelay\KatalonData\Bootstrap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{11A59C1D-CBA4-4554-87DA-448528D6B305}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F05834B-927F-4BAF-A5F2-37F83D71699F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="5" firstSheet="2" windowHeight="12456" windowWidth="23256" xWindow="-108" xr2:uid="{354FC140-4496-4D7F-AB69-566E59F6C646}" yWindow="-108"/>
+    <workbookView xWindow="792" yWindow="1572" windowWidth="17280" windowHeight="9972" firstSheet="2" activeTab="5" xr2:uid="{354FC140-4496-4D7F-AB69-566E59F6C646}"/>
   </bookViews>
   <sheets>
-    <sheet name="CreateUser" r:id="rId1" sheetId="1"/>
-    <sheet name="FindUser" r:id="rId2" sheetId="7"/>
-    <sheet name="ModifyUser" r:id="rId3" sheetId="18"/>
-    <sheet name="ModifyUserPwd" r:id="rId4" sheetId="19"/>
-    <sheet name="FindCaseUser" r:id="rId5" sheetId="20"/>
-    <sheet name="AddDeleteRole" r:id="rId6" sheetId="16"/>
-    <sheet name="SearchRole" r:id="rId7" sheetId="17"/>
+    <sheet name="CreateUser" sheetId="1" r:id="rId1"/>
+    <sheet name="FindUser" sheetId="7" r:id="rId2"/>
+    <sheet name="ModifyUser" sheetId="18" r:id="rId3"/>
+    <sheet name="ModifyUserPwd" sheetId="19" r:id="rId4"/>
+    <sheet name="FindCaseUser" sheetId="20" r:id="rId5"/>
+    <sheet name="AddDeleteRole" sheetId="16" r:id="rId6"/>
+    <sheet name="SearchRole" sheetId="17" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="65">
   <si>
     <t>Notes</t>
   </si>
@@ -148,385 +148,94 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>Thu Nov 20 15:06:26 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 15:07:04 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 15:07:46 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 15:09:20 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 15:10:39 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 19:00:09 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 19:00:56 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 19:01:35 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 19:02:22 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 19:02:53 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 19:03:49 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 19:05:16 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 21:26:52 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 20 21:54:04 IST 2025</t>
-  </si>
-  <si>
-    <t>Prod Role</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Thu Nov 20 21:56:43 IST 2025</t>
-  </si>
-  <si>
-    <t>Tue Feb 17 23:59:01 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 17 23:59:42 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 18 00:00:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 18 00:00:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 18 00:01:29 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 18 00:02:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 18 00:03:09 IST 2026</t>
-  </si>
-  <si>
-    <t>Sun Feb 22 23:01:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Sun Feb 22 23:02:48 IST 2026</t>
-  </si>
-  <si>
-    <t>Sun Feb 22 23:03:21 IST 2026</t>
-  </si>
-  <si>
-    <t>Sun Feb 22 23:03:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Sun Feb 22 23:04:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Sun Feb 22 23:05:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Sun Feb 22 23:06:36 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 00:13:41 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 00:15:23 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 00:16:42 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 00:17:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 00:18:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 00:18:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 00:30:22 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 20:22:21 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 21:36:42 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 21:38:13 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 24 21:39:45 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 25 22:29:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 25 22:30:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 25 22:31:22 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 25 22:32:21 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 25 22:32:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 25 22:34:09 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 25 22:35:35 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 06:54:27 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 06:55:19 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 06:55:54 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 06:56:22 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 06:56:53 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 06:57:40 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 06:58:57 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 08:33:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 22:24:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 22:25:30 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 22:26:11 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 22:26:57 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 22:27:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 22:28:31 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 26 22:29:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:39:25 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:41:28 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:42:57 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:44:36 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:46:11 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:47:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:59:48 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 21:19:24 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 21:20:47 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 21:21:43 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 21:22:25 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 21:23:25 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 21:24:53 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 21:26:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 00:41:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 08:06:47 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 08:07:36 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 08:08:06 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 08:08:48 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 08:09:23 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 08:10:31 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 05 08:11:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 00:50:31 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 00:51:23 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 00:51:56 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 00:52:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 00:53:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 00:54:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 00:55:16 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 06:30:21 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 06:31:22 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 06:32:12 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 06:33:00 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 06:33:39 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 06:34:39 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 06:35:59 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 22 20:38:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 22 20:39:40 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 22 20:40:24 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 22 20:41:09 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 22 20:41:46 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 22 20:43:27 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 22 20:44:46 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri May 08 23:30:01 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri May 08 23:31:11 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri May 08 23:31:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri May 08 23:32:28 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri May 08 23:33:00 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri May 08 23:33:54 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri May 08 23:35:20 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon May 11 18:58:08 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon May 11 18:59:30 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon May 11 19:04:12 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon May 11 21:58:15 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue May 12 19:21:34 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue May 12 19:58:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 16 23:39:10 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 16 23:39:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 16 23:40:31 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 16 23:41:11 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 16 23:41:46 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 16 23:42:42 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 16 23:43:48 IST 2026</t>
+    <t>Thu Jul 02 19:23:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Jul 02 19:24:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Jul 02 19:24:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Jul 02 19:25:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Jul 02 19:25:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Jul 02 19:26:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Jul 02 19:27:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 16:46:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 16:48:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 16:52:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 16:53:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 20:32:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 20:35:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 20:37:28 IST 2026</t>
+  </si>
+  <si>
+    <t>New Prod Role</t>
+  </si>
+  <si>
+    <t>Mon Jul 06 21:33:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:18:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:19:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:20:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:20:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:21:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:22:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 07 16:23:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Jul 08 06:16:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Jul 08 06:17:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Jul 08 06:18:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Jul 08 06:19:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Jul 08 06:19:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Jul 08 06:20:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Jul 08 06:21:42 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -576,21 +285,21 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -607,10 +316,10 @@
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -645,7 +354,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin panose="020F0302020204030204" typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -697,7 +406,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin panose="020F0502020204030204" typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -808,21 +517,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="6350">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -839,7 +548,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -891,15 +600,15 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" name="Office 2013 - 2022 Theme" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E041308-6561-4EE5-9DD4-5DDA2695E487}">
-  <dimension ref="A1:O4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E041308-6561-4EE5-9DD4-5DDA2695E487}">
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.5546875" collapsed="true"/>
@@ -918,7 +627,7 @@
     <col min="15" max="16384" style="1" width="9.109375" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -963,17 +672,17 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>157</v>
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>8</v>
@@ -987,10 +696,10 @@
       <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="1" t="s">
         <v>15</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -998,17 +707,11 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
       <c r="K4" s="2"/>
-      <c r="L4"/>
-      <c r="M4"/>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -1016,8 +719,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D7D96D8-F32A-42CB-8719-B4A22D28EC0D}">
-  <dimension ref="A1:L13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D7D96D8-F32A-42CB-8719-B4A22D28EC0D}">
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="19.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.5546875" collapsed="true"/>
@@ -1033,7 +736,7 @@
     <col min="12" max="16384" style="1" width="19.33203125" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="28.8" r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1069,17 +772,17 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>158</v>
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>8</v>
@@ -1094,69 +797,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3"/>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5"/>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7"/>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8"/>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9"/>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10"/>
-      <c r="B10"/>
-      <c r="C10"/>
-      <c r="D10"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11"/>
-      <c r="B11"/>
-      <c r="C11"/>
-      <c r="D11"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12"/>
-      <c r="B12"/>
-      <c r="C12"/>
-      <c r="D12"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13"/>
-      <c r="B13"/>
-      <c r="C13"/>
-      <c r="D13"/>
-    </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -1164,14 +807,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28ECF6F8-94D7-41D5-B6FF-650248E68667}">
-  <dimension ref="A1:O2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28ECF6F8-94D7-41D5-B6FF-650248E68667}">
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="8" customWidth="true" width="30.109375" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1216,17 +859,17 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>159</v>
+      <c r="A2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>39</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
@@ -1243,10 +886,10 @@
       <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>15</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -1254,13 +897,13 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5380E685-D2A4-4DCA-A76F-EFBA3980BCE7}">
-  <dimension ref="A1:O2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5380E685-D2A4-4DCA-A76F-EFBA3980BCE7}">
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" customWidth="true" width="22.33203125" collapsed="true"/>
@@ -1271,98 +914,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" t="s" s="0">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>160</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="A2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="H2" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="0">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ECF5EAC-3F98-4000-BEA2-335F903FE34F}">
-  <dimension ref="A1:M2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ECF5EAC-3F98-4000-BEA2-335F903FE34F}">
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="9" customWidth="true" width="22.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="28.8" r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1400,18 +1043,18 @@
         <v>12</v>
       </c>
     </row>
-    <row ht="28.8" r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>161</v>
+    <row r="2" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>41</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
@@ -1433,13 +1076,13 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A53983D-C89C-4548-8A02-C36CB8EC5C28}">
-  <dimension ref="A1:J5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A53983D-C89C-4548-8A02-C36CB8EC5C28}">
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="3" width="6.5546875" collapsed="true"/>
@@ -1450,7 +1093,7 @@
     <col min="10" max="16384" style="3" width="9.109375" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="28.8" r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1480,17 +1123,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>155</v>
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>8</v>
@@ -1505,32 +1148,14 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3"/>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5"/>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
-    </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCABF931-E9E5-40BE-B844-C9FC3C47A38B}">
-  <dimension ref="A1:J5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCABF931-E9E5-40BE-B844-C9FC3C47A38B}">
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" style="3" width="9.109375" collapsed="true"/>
@@ -1541,7 +1166,7 @@
     <col min="10" max="16384" style="3" width="9.109375" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="28.8" r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1571,17 +1196,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>156</v>
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>8</v>
@@ -1596,25 +1221,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3"/>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5"/>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
-    </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>